<commit_message>
Record transit/T1 status as unresolved
No transit declaration is among the documents. The only mention in the
whole thread is Hitachi asking DSV to confirm the shipment moves without
T1; DSV never answered that question and closed with having no further
documents. The Dispozice form leaves the T1 box and the office of
destination blank.

The single MRN in the correspondence, 26GB000246SZVJOHJ0, is described
only as "SCP MRN". Since the UK is a party to the Common Transit
Convention, a T1 opened there also carries a GB prefix, so the prefix
alone does not establish that this is an export rather than a transit
declaration. Records the questions DSV needs to answer in writing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016ex1XUHp1Tm7yTQTPEjtdL
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Energy_129689.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Energy_129689.xlsx
@@ -5176,7 +5176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B90"/>
+  <dimension ref="A1:B100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -5776,95 +5776,164 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="31" t="inlineStr">
-        <is>
-          <t>7) PROVOZNÍ POZNÁMKY K ZÁSILCE</t>
-        </is>
-      </c>
-      <c r="B79" s="32" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="30" customHeight="1">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t>7) TRANZIT / T1 – NEMÁME, STAV NEPOTVRZEN</t>
+        </is>
+      </c>
+      <c r="B79" s="26" t="inlineStr">
+        <is>
+          <t>NEVYŘEŠENO</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="45" customHeight="1">
       <c r="A80" s="22" t="inlineStr">
         <is>
-          <t>Přeprava: DSV Road s.r.o. (Alena Miková), zásilka GBPFT608004151 / MSA850/012. Vývozní MRN (SCP): 26GB000246SZVJOHJ0.</t>
+          <t>❌ Mezi doloženými doklady NENÍ žádné tranzitní celní prohlášení (T1) ani jiný tranzitní doklad. K dispozici máme pouze: Customs Invoice 129689, Packing Note, Export Declaration Instruction Sheet 1400045712, Supplier's Declaration (export control), PO 4502372958 a nevyplněný formulář Dispozice IMPORT.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="22" t="inlineStr">
         <is>
-          <t>Pan Jahnholz uvádí, že jde o přepravu BEZ T1, a žádá o potvrzení – ověřte, zda k zásilce existuje tranzitní doklad, nebo zda se clí přímo na základě vývozního MRN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="30" customHeight="1">
+          <t xml:space="preserve">V celé e-mailové korespondenci se T1 zmiňuje jedinkrát – pan Jahnholz (Hitachi Energy) 11.09.2026: „Pokud vím, jedná se o přepravu bez T1; prosím o potvrzení.“ </t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="45" customHeight="1">
       <c r="A82" s="22" t="inlineStr">
         <is>
+          <t>⚠ TOTO POTVRZENÍ NIKDY NEPŘIŠLO. DSV (paní Miková) na dotaz k T1 neodpověděla; její poslední zpráva zní „já více dokladů k dispozici nemám“. Stav tranzitu je tedy otevřený – nelze vycházet z toho, že T1 neexistuje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="22" t="inlineStr">
+        <is>
+          <t>Jediné MRN v korespondenci je 26GB000246SZVJOHJ0, které DSV označuje jako „SCP MRN“. Z označení nelze určit, zda jde o britské vývozní celní prohlášení, nebo o tranzitní prohlášení.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="45" customHeight="1">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t>⚠ POZOR: Spojené království je smluvní stranou Úmluvy o společném tranzitním režimu, takže i T1 otevřené v GB nese MRN s předponou GB. Prefix „26GB…“ tedy sám o sobě NEDOKAZUJE, že jde o vývozní a nikoli tranzitní doklad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="60" customHeight="1">
+      <c r="A85" s="22" t="inlineStr">
+        <is>
+          <t>➤ PROČ NA TOM ZÁLEŽÍ: pokud T1 existuje, musí je Maurice Ward u celního úřadu určení řádně a včas ukončit a JSD musí na tento předchozí doklad odkazovat. Pokud T1 neexistuje, muselo být zboží propuštěno do celního režimu již v místě vstupu do EU – a to místo je dosud „unknown“. Ani jedna varianta zatím není doložena.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>➤ Formulář Dispozice IMPORT má kolonku „Tranzitní celní prohlášení (T1): ANO / NE“ i „Celní úřad určení“ NEVYPLNĚNÉ, včetně závazku „V případě tohoto režimu se zavazujeme T1 včas a řádně ukončit“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="45" customHeight="1">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>➤ DOTAZ NA DSV (paní Miková) – vyžádat písemně: (1) bylo k zásilce otevřeno tranzitní prohlášení T1, ano či ne? (2) pokud ano, jaké je MRN tranzitu a který je celní úřad určení? (3) co přesně je MRN 26GB000246SZVJOHJ0 – vývozní, nebo tranzitní prohlášení? (4) kde zásilka vstoupila na celní území EU?</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="31" t="inlineStr">
+        <is>
+          <t>8) PROVOZNÍ POZNÁMKY K ZÁSILCE</t>
+        </is>
+      </c>
+      <c r="B89" s="32" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="22" t="inlineStr">
+        <is>
+          <t>Přeprava: DSV Road s.r.o. (Alena Miková), zásilka GBPFT608004151 / MSA850/012. Vývozní MRN (SCP): 26GB000246SZVJOHJ0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="22" t="inlineStr">
+        <is>
+          <t>Tranzit / T1: viz samostatná sekce 7 – stav není potvrzen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="22" t="inlineStr">
+        <is>
           <t>DSV k zásilce neměla dovozní fakturu (měla pouze objednávku a export declaration sheet); fakturu 129689 dodala přímo Hitachi Energy (Mathias Jahnholz) – ta je podkladem tohoto souhrnu.</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="15" customHeight="1">
-      <c r="A83" s="22" t="inlineStr">
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="22" t="inlineStr">
         <is>
           <t>Vykládka: 14./15.09.2026, Trutnov, Průmyslová 137. Kontakt příjemce: Monika Lutterová, +420 704 844 676.</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="30" customHeight="1">
-      <c r="A84" s="22" t="inlineStr">
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="22" t="inlineStr">
         <is>
           <t>Vývozní kontrola: Supplier's Declaration concerning Export Control potvrzuje u VŠECH položek Dual-Use = No, vojenské zboží N/A, ITAR N/A – zboží nepodléhá vývozním omezením.</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="45" customHeight="1">
-      <c r="A85" s="22" t="inlineStr">
+    <row r="95" ht="45" customHeight="1">
+      <c r="A95" s="22" t="inlineStr">
         <is>
           <t>PO 4502372958 (19.08.2026) = objednávka přepravy u DSV Road Ltd, 487,10 GBP, dodání 28.08.2026. Obsahuje rovněž prohlášení dodavatele, že zboží NENÍ ruského původu a neobsahuje železné ani ocelové výrobky ruského původu – využitelné k doložení souladu se sankčním režimem (čl. 3g nařízení 833/2014).</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="60" customHeight="1">
-      <c r="A86" s="22" t="inlineStr">
+    <row r="96" ht="60" customHeight="1">
+      <c r="A96" s="22" t="inlineStr">
         <is>
           <t>„Dispozice IMPORT“ je nevyplněný formulář objednávky celních služeb Maurice Ward. Požaduje přesně tyto údaje: český popis zboží, TARIC, hodnotu, nákladové kusy, hrubou a čistou hmotnost – všechny jsou na listu „Souhrn HS“. Formulář je dosud nevyplněný a nepodepsaný; před odbavením jej nechte dovozce doplnit a podepsat.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="29" t="inlineStr">
-        <is>
-          <t>8) POZNÁMKA K POPISŮM V ČEŠTINĚ</t>
-        </is>
-      </c>
-      <c r="B88" s="30" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
+          <t>9) POZNÁMKA K POPISŮM V ČEŠTINĚ</t>
+        </is>
+      </c>
+      <c r="B98" s="30" t="inlineStr">
         <is>
           <t>POZOR</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="22" t="inlineStr">
+    <row r="99" ht="30" customHeight="1">
+      <c r="A99" s="22" t="inlineStr">
         <is>
           <t>Zdrojové doklady (faktura, packing note, export declaration, supplier's declaration) jsou POUZE v angličtině – český popis zboží v nich není k dispozici.</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="45" customHeight="1">
-      <c r="A90" s="22" t="inlineStr">
+    <row r="100" ht="45" customHeight="1">
+      <c r="A100" s="22" t="inlineStr">
         <is>
           <t>Sloupec „Popis zboží (CZ)“ na listu „Souhrn HS“ je proto překlad podle znění kombinované nomenklatury k danému HS kódu, nikoli převzatý údaj ze zdrojového dokladu. Původní anglický popis je zachován ve vedlejším sloupci.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="52">
+  <mergeCells count="60">
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A92:B92"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A82:B82"/>
     <mergeCell ref="A73:B73"/>
@@ -5872,15 +5941,17 @@
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A94:B94"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A87:B87"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A90:B90"/>
+    <mergeCell ref="A99:B99"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="A84:B84"/>
-    <mergeCell ref="A89:B89"/>
     <mergeCell ref="A74:B74"/>
     <mergeCell ref="A80:B80"/>
     <mergeCell ref="A18:B18"/>
@@ -5888,6 +5959,7 @@
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A86:B86"/>
+    <mergeCell ref="A95:B95"/>
     <mergeCell ref="A76:B76"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A71:B71"/>
@@ -5901,15 +5973,19 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A91:B91"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A100:B100"/>
     <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A96:B96"/>
     <mergeCell ref="A72:B72"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A81:B81"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A93:B93"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A83:B83"/>
     <mergeCell ref="A44:B44"/>

</xml_diff>